<commit_message>
feat: implement database reset seed script and add production docker configuration
</commit_message>
<xml_diff>
--- a/Sections.xlsx
+++ b/Sections.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MrF41C0N\Desktop\GitHub\AIMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B8C9EC-4A01-4856-881B-39D449115333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B32D38-1C44-4314-9224-5F0D91042698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{01611521-4A96-437A-A59E-2BFE4F41F415}"/>
   </bookViews>
@@ -42,101 +42,100 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>SL No</t>
   </si>
   <si>
-    <t>Designations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	Asst. Accounts Officer</t>
-  </si>
-  <si>
-    <t>Accountant</t>
-  </si>
-  <si>
-    <t>Assistant Supervisor</t>
-  </si>
-  <si>
-    <t>Canteen Attendant</t>
-  </si>
-  <si>
-    <t>Canteen Attendant (Outsourced)</t>
-  </si>
-  <si>
-    <t>Casual Worker Tripura</t>
-  </si>
-  <si>
-    <t>Clerk Typist</t>
-  </si>
-  <si>
-    <t>Consultant Accountant</t>
-  </si>
-  <si>
-    <t>Data Entry Operator (Outsourced)</t>
-  </si>
-  <si>
-    <t>Data Entry Operator Gr B</t>
-  </si>
-  <si>
-    <t>Data Entry Operator Gr A</t>
-  </si>
-  <si>
-    <t>Halwai</t>
-  </si>
-  <si>
-    <t>Junior Translator</t>
-  </si>
-  <si>
-    <t>Multi Task Staff</t>
-  </si>
-  <si>
-    <t>Multi Tasking Staff (Outsourced)</t>
-  </si>
-  <si>
-    <t>Outsourced Canteen Manager</t>
-  </si>
-  <si>
-    <t>Roll out Support Engineer</t>
-  </si>
-  <si>
-    <t>Senior Accounts Officer</t>
-  </si>
-  <si>
-    <t>Senior Accountant</t>
-  </si>
-  <si>
-    <t>Senior Deputy Accountant General</t>
-  </si>
-  <si>
-    <t>Senior Hindi Translator</t>
-  </si>
-  <si>
-    <t>Stenographer</t>
-  </si>
-  <si>
-    <t>Stenographer (Outsourced)</t>
-  </si>
-  <si>
-    <t>Supervisor</t>
-  </si>
-  <si>
-    <t>Canteen Clerk</t>
-  </si>
-  <si>
-    <t>Accountant General (A&amp;E)</t>
-  </si>
-  <si>
-    <t>Hindi Translator</t>
+    <t>VLCS</t>
+  </si>
+  <si>
+    <t>IT CELL</t>
+  </si>
+  <si>
+    <t>Record Section</t>
+  </si>
+  <si>
+    <t>AG Cell</t>
+  </si>
+  <si>
+    <t>Sr.DAG Cell</t>
+  </si>
+  <si>
+    <t>Book Section</t>
+  </si>
+  <si>
+    <t>AC section</t>
+  </si>
+  <si>
+    <t>FA Cell</t>
+  </si>
+  <si>
+    <t>Establishment</t>
+  </si>
+  <si>
+    <t>CA Section</t>
+  </si>
+  <si>
+    <t>TMC</t>
+  </si>
+  <si>
+    <t>EDP-GPF</t>
+  </si>
+  <si>
+    <t>ITA Section</t>
+  </si>
+  <si>
+    <t>Senior Deputy Accountant General (Sr. DAG), Tripura</t>
+  </si>
+  <si>
+    <t>A.G. Sectariat</t>
+  </si>
+  <si>
+    <t>Departmental Canteen</t>
+  </si>
+  <si>
+    <t>EDP-PF</t>
+  </si>
+  <si>
+    <t>Hindi Anubhag</t>
+  </si>
+  <si>
+    <t>Legal Section</t>
+  </si>
+  <si>
+    <t>Pension-II</t>
+  </si>
+  <si>
+    <t>Pension-III</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pension -I </t>
+  </si>
+  <si>
+    <t>PAO  (Local)</t>
+  </si>
+  <si>
+    <t>HoD, Accountant General (A&amp;E), Tripura</t>
+  </si>
+  <si>
+    <t>Section Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -164,46 +163,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -554,245 +527,222 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F15EB73B-0606-483E-A81A-370F376E0223}">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
+      <c r="B1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>27</v>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>4</v>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>5</v>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>6</v>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>26</v>
+      <c r="B8" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
-        <v>7</v>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
-        <v>8</v>
+      <c r="B10" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>9</v>
+      <c r="B11" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
         <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>16</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>17</v>
-      </c>
-      <c r="B17" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="B21" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>22</v>
-      </c>
-      <c r="B22" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>23</v>
-      </c>
-      <c r="B23" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>24</v>
-      </c>
-      <c r="B24" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>25</v>
-      </c>
-      <c r="B25" t="s">
-        <v>22</v>
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>26</v>
-      </c>
-      <c r="B26" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>27</v>
-      </c>
-      <c r="B27" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>28</v>
-      </c>
-      <c r="B28" t="s">
-        <v>25</v>
-      </c>
+      <c r="B26"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{F15EB73B-0606-483E-A81A-370F376E0223}"/>
-  <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="2" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B7 B9:B1048576">
+  <conditionalFormatting sqref="B1:B3 B5:B25 B27:B1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
+  <conditionalFormatting sqref="B4">
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>